<commit_message>
Add profile system, knowledge separation, worksheet generation, improved AI personality
</commit_message>
<xml_diff>
--- a/knowledge/eskool.xlsx
+++ b/knowledge/eskool.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yeghia\whatsapp-ai-bot\knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29AC84A8-751E-467E-89D9-444CCB3A0A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8E351D-06E6-40F9-A04C-37F61D467B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Issue</t>
   </si>
@@ -32,11 +32,6 @@
   </si>
   <si>
     <t>Cannot log in</t>
-  </si>
-  <si>
-    <t>1. Go to www.aechs.com
-2. Enter your username and password
-3. If forgotten, contact Mr. Yeghia to reset</t>
   </si>
   <si>
     <t>Teacher usernames are usually firstname.lastname</t>
@@ -50,9 +45,6 @@
 3. Check WiFi connection</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Grades not saving</t>
   </si>
   <si>
@@ -64,26 +56,44 @@
     <t>Cannot see students</t>
   </si>
   <si>
-    <t>Make sure you are in the correct class/section. Contact Mr. Yeghia if section is missing</t>
-  </si>
-  <si>
     <t>Forgot password</t>
   </si>
   <si>
-    <t>Contact Mr. Yeghia on 96170688510 to reset</t>
+    <t>Cannot publish meeting — Zoom not configured</t>
+  </si>
+  <si>
+    <t>The organizer's Zoom account is not linked to ESkool. Go to your profile settings in ESkool and connect your Zoom account. If the issue persists, contact Mr. Jawad for ESkool support.</t>
+  </si>
+  <si>
+    <t>Error message: The organizer's Zoom account is not configured properly</t>
+  </si>
+  <si>
+    <t>1. Go to www.aechs.com
+2. Enter your username and password
+3. If forgotten, contact Mr. Jawad to reset</t>
+  </si>
+  <si>
+    <t>Make sure you are in the correct class/section. Contact Mr. Jawad if section is missing</t>
+  </si>
+  <si>
+    <t>Contact Mr. Jawad on 96170688510 to reset</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -94,7 +104,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -102,12 +112,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,15 +478,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="90" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="43.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -466,65 +497,61 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C7" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C6" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Structured JSON architecture, profile system, PDF worksheet generation, multi-page support
</commit_message>
<xml_diff>
--- a/knowledge/eskool.xlsx
+++ b/knowledge/eskool.xlsx
@@ -1,104 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yeghia\whatsapp-ai-bot\knowledge\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8E351D-06E6-40F9-A04C-37F61D467B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="eskool" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eskool" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t>Issue</t>
-  </si>
-  <si>
-    <t>Solution</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Cannot log in</t>
-  </si>
-  <si>
-    <t>Teacher usernames are usually firstname.lastname</t>
-  </si>
-  <si>
-    <t>Page not loading</t>
-  </si>
-  <si>
-    <t>1. Clear browser cache (Ctrl+Shift+Delete)
-2. Try a different browser
-3. Check WiFi connection</t>
-  </si>
-  <si>
-    <t>Grades not saving</t>
-  </si>
-  <si>
-    <t>1. Check internet connection
-2. Do not use browser back button
-3. Always click Save before leaving page</t>
-  </si>
-  <si>
-    <t>Cannot see students</t>
-  </si>
-  <si>
-    <t>Forgot password</t>
-  </si>
-  <si>
-    <t>Cannot publish meeting — Zoom not configured</t>
-  </si>
-  <si>
-    <t>The organizer's Zoom account is not linked to ESkool. Go to your profile settings in ESkool and connect your Zoom account. If the issue persists, contact Mr. Jawad for ESkool support.</t>
-  </si>
-  <si>
-    <t>Error message: The organizer's Zoom account is not configured properly</t>
-  </si>
-  <si>
-    <t>1. Go to www.aechs.com
-2. Enter your username and password
-3. If forgotten, contact Mr. Jawad to reset</t>
-  </si>
-  <si>
-    <t>Make sure you are in the correct class/section. Contact Mr. Jawad if section is missing</t>
-  </si>
-  <si>
-    <t>Contact Mr. Jawad on 96170688510 to reset</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <sz val="10"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -113,46 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -477,78 +457,126 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="90" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.375" bestFit="1" customWidth="1"/>
+    <col width="17.75" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="90" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="43.375" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>13</v>
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Solution</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cannot log in</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1. Go to www.aechs.com
+2. Enter your username and password
+3. If forgotten, contact Mr. Yeghia to reset</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Teacher usernames are usually firstname.lastname</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Page not loading</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1. Clear browser cache (Ctrl+Shift+Delete)
+2. Try a different browser
+3. Check WiFi connection</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Grades not saving</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1. Check internet connection
+2. Do not use browser back button
+3. Always click Save before leaving page</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cannot see students</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Make sure you are in the correct class/section. Contact Mr. Yeghia if section is missing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Forgot password</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Contact Mr. Yeghia on 96170688510 to reset</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Cannot publish meeting — Zoom not configured</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>The organizer's Zoom account is not linked to ESkool. Go to your profile settings in ESkool and connect your Zoom account. If the issue persists, contact Mr. Jawad for ESkool support.</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Error message: The organizer's Zoom account is not configured properly</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update core files, knowledge base, and assets
</commit_message>
<xml_diff>
--- a/knowledge/eskool.xlsx
+++ b/knowledge/eskool.xlsx
@@ -1,43 +1,58 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eskool" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="eskool" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,94 +60,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -457,129 +396,95 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17.75" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="90" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="43.375" bestFit="1" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Issue</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Solution</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Cannot log in</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1. Go to www.aechs.com
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Issue</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>Cannot log in</v>
+      </c>
+      <c r="B2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to www.aechs.com
 2. Enter your username and password
-3. If forgotten, contact Mr. Yeghia to reset</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Teacher usernames are usually firstname.lastname</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page not loading</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1. Clear browser cache (Ctrl+Shift+Delete)
+3. If forgotten, contact Mr. Yeghia to reset</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Teacher usernames are usually firstname.lastname</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>Page not loading</v>
+      </c>
+      <c r="B3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Clear browser cache (Ctrl+Shift+Delete)
 2. Try a different browser
-3. Check WiFi connection</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Grades not saving</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1. Check internet connection
+3. Check WiFi connection</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>Grades not saving</v>
+      </c>
+      <c r="B4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Check internet connection
 2. Do not use browser back button
-3. Always click Save before leaving page</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Cannot see students</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Make sure you are in the correct class/section. Contact Mr. Yeghia if section is missing</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Forgot password</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Contact Mr. Yeghia on 96170688510 to reset</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+3. Always click Save before leaving page</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Cannot see students</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Make sure you are in the correct class/section. Contact Mr. Yeghia if section is missing</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Forgot password</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Contact Mr. Yeghia on 96170688510 to reset</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Cannot publish meeting — Zoom not configured</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>The organizer's Zoom account is not linked to ESkool. Go to your profile settings in ESkool and connect your Zoom account. If the issue persists, contact Mr. Jawad for ESkool support.</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>Error message: The organizer's Zoom account is not configured properly</t>
-        </is>
+      <c r="A7" t="str">
+        <v>Cannot publish meeting — Zoom not configured</v>
+      </c>
+      <c r="B7" t="str">
+        <v>The organizer's Zoom account is not linked to ESkool. Go to your profile settings in ESkool and connect your Zoom account. If the issue persists, contact Mr. Jawad for ESkool support.</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Error message: The organizer's Zoom account is not configured properly</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>